<commit_message>
Make retention gifts one-time and improve welfare UI
Limit retention gifts to the first configured minutes of each session and persist one-time claims. Close other dialogs before showing gifts, refresh welfare countdowns, and keep item descriptions visible independently of the strength bar.
</commit_message>
<xml_diff>
--- a/配置文档/ActivityConfig.xlsx
+++ b/配置文档/ActivityConfig.xlsx
@@ -694,10 +694,10 @@
     <s:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <s:alignment vertical="center"/>
     </s:xf>
+    <s:xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <s:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <s:alignment horizontal="center" vertical="center"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <s:xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <s:alignment horizontal="center" vertical="top" wrapText="1"/>
     </s:xf>
@@ -1101,12 +1101,12 @@
   <s:dimension ref="A1:F5"/>
   <s:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="4" outlineLevelCol="5"/>
   <s:cols>
-    <s:col width="16.6666666666667" customWidth="1" style="2" min="1" max="1"/>
-    <s:col width="29" customWidth="1" style="2" min="2" max="2"/>
-    <s:col width="27.3333333333333" customWidth="1" style="2" min="3" max="3"/>
-    <s:col width="24.8916666666667" customWidth="1" style="2" min="4" max="4"/>
-    <s:col width="22.8916666666667" customWidth="1" style="2" min="5" max="5"/>
-    <s:col width="23.775" customWidth="1" style="2" min="6" max="6"/>
+    <s:col width="16.6666666666667" customWidth="1" style="1" min="1" max="1"/>
+    <s:col width="29" customWidth="1" style="1" min="2" max="2"/>
+    <s:col width="27.3333333333333" customWidth="1" style="1" min="3" max="3"/>
+    <s:col width="24.8916666666667" customWidth="1" style="1" min="4" max="4"/>
+    <s:col width="22.8916666666667" customWidth="1" style="1" min="5" max="5"/>
+    <s:col width="23.775" customWidth="1" style="1" min="6" max="6"/>
   </s:cols>
   <s:sheetData>
     <s:row r="1">
@@ -1261,7 +1261,7 @@
       </s:c>
       <s:c r="F5" s="0" t="inlineStr">
         <s:is>
-          <s:t>ESC 挽留礼包：提示时长与在线奖励引用；与福利页共享每日领取记录，不额外发奖</s:t>
+          <s:t>ESC 一次性挽留礼包：仅本次进服后的指定分钟数之内提示，每个玩家永久只能领取一次</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -1283,114 +1283,114 @@
   <s:dimension ref="A1:G8"/>
   <s:sheetFormatPr baseColWidth="8" defaultColWidth="8.891666666666669" defaultRowHeight="13.5" outlineLevelRow="7" outlineLevelCol="6"/>
   <s:cols>
-    <s:col width="16.9416666666667" customWidth="1" style="2" min="2" max="2"/>
-    <s:col width="35.8916666666667" customWidth="1" style="2" min="3" max="3"/>
-    <s:col width="17.8333333333333" customWidth="1" style="2" min="4" max="5"/>
-    <s:col width="32.1416666666667" customWidth="1" style="2" min="6" max="6"/>
-    <s:col width="16.3416666666667" customWidth="1" style="2" min="7" max="7"/>
+    <s:col width="16.9416666666667" customWidth="1" style="1" min="2" max="2"/>
+    <s:col width="35.8916666666667" customWidth="1" style="1" min="3" max="3"/>
+    <s:col width="17.8333333333333" customWidth="1" style="1" min="4" max="5"/>
+    <s:col width="32.1416666666667" customWidth="1" style="1" min="6" max="6"/>
+    <s:col width="16.3416666666667" customWidth="1" style="1" min="7" max="7"/>
   </s:cols>
   <s:sheetData>
     <s:row r="1">
-      <s:c r="A1" s="1" t="inlineStr">
+      <s:c r="A1" s="2" t="inlineStr">
         <s:is>
           <s:t>索引</s:t>
         </s:is>
       </s:c>
-      <s:c r="B1" s="1" t="inlineStr">
+      <s:c r="B1" s="2" t="inlineStr">
         <s:is>
           <s:t>任务类型</s:t>
         </s:is>
       </s:c>
-      <s:c r="C1" s="1" t="inlineStr">
+      <s:c r="C1" s="2" t="inlineStr">
         <s:is>
           <s:t>名字</s:t>
         </s:is>
       </s:c>
-      <s:c r="D1" s="1" t="inlineStr">
+      <s:c r="D1" s="2" t="inlineStr">
         <s:is>
           <s:t>描述</s:t>
         </s:is>
       </s:c>
-      <s:c r="E1" s="1" t="inlineStr">
+      <s:c r="E1" s="2" t="inlineStr">
         <s:is>
           <s:t>目标值</s:t>
         </s:is>
       </s:c>
-      <s:c r="F1" s="1" t="inlineStr">
+      <s:c r="F1" s="2" t="inlineStr">
         <s:is>
           <s:t>奖励</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="2">
-      <s:c r="A2" s="1" t="inlineStr">
+      <s:c r="A2" s="2" t="inlineStr">
         <s:is>
           <s:t>Index</s:t>
         </s:is>
       </s:c>
-      <s:c r="B2" s="1" t="inlineStr">
+      <s:c r="B2" s="2" t="inlineStr">
         <s:is>
           <s:t>Type</s:t>
         </s:is>
       </s:c>
-      <s:c r="C2" s="1" t="inlineStr">
+      <s:c r="C2" s="2" t="inlineStr">
         <s:is>
           <s:t>Name</s:t>
         </s:is>
       </s:c>
-      <s:c r="D2" s="1" t="inlineStr">
+      <s:c r="D2" s="2" t="inlineStr">
         <s:is>
           <s:t>Desc</s:t>
         </s:is>
       </s:c>
-      <s:c r="E2" s="1" t="inlineStr">
+      <s:c r="E2" s="2" t="inlineStr">
         <s:is>
           <s:t>Target</s:t>
         </s:is>
       </s:c>
-      <s:c r="F2" s="1" t="inlineStr">
+      <s:c r="F2" s="2" t="inlineStr">
         <s:is>
           <s:t>Rewards</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="3">
-      <s:c r="A3" s="1" t="inlineStr">
+      <s:c r="A3" s="2" t="inlineStr">
         <s:is>
           <s:t>number</s:t>
         </s:is>
       </s:c>
-      <s:c r="B3" s="1" t="inlineStr">
+      <s:c r="B3" s="2" t="inlineStr">
         <s:is>
           <s:t>string</s:t>
         </s:is>
       </s:c>
-      <s:c r="C3" s="1" t="inlineStr">
+      <s:c r="C3" s="2" t="inlineStr">
         <s:is>
           <s:t>string</s:t>
         </s:is>
       </s:c>
-      <s:c r="D3" s="1" t="inlineStr">
+      <s:c r="D3" s="2" t="inlineStr">
         <s:is>
           <s:t>string</s:t>
         </s:is>
       </s:c>
-      <s:c r="E3" s="1" t="inlineStr">
+      <s:c r="E3" s="2" t="inlineStr">
         <s:is>
           <s:t>number_option</s:t>
         </s:is>
       </s:c>
-      <s:c r="F3" s="1" t="inlineStr">
+      <s:c r="F3" s="2" t="inlineStr">
         <s:is>
           <s:t>kv_string_array</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="4">
-      <s:c r="A4" s="1" t="n">
+      <s:c r="A4" s="2" t="n">
         <s:v>1</s:v>
       </s:c>
-      <s:c r="B4" s="1" t="inlineStr">
+      <s:c r="B4" s="2" t="inlineStr">
         <s:is>
           <s:t>GetItem</s:t>
         </s:is>
@@ -1405,25 +1405,25 @@
           <s:t>Pick up 50 items</s:t>
         </s:is>
       </s:c>
-      <s:c r="E4" s="1" t="n">
+      <s:c r="E4" s="2" t="n">
         <s:v>50</s:v>
       </s:c>
-      <s:c r="F4" s="1" t="inlineStr">
+      <s:c r="F4" s="2" t="inlineStr">
         <s:is>
           <s:t>{Type=Gem, Count=3}</s:t>
         </s:is>
       </s:c>
-      <s:c r="G4" s="1" t="inlineStr">
+      <s:c r="G4" s="2" t="inlineStr">
         <s:is>
           <s:t>3钻石</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="5">
-      <s:c r="A5" s="1" t="n">
+      <s:c r="A5" s="2" t="n">
         <s:v>2</s:v>
       </s:c>
-      <s:c r="B5" s="1" t="inlineStr">
+      <s:c r="B5" s="2" t="inlineStr">
         <s:is>
           <s:t>GetItem</s:t>
         </s:is>
@@ -1438,25 +1438,25 @@
           <s:t>Pick up 80 items</s:t>
         </s:is>
       </s:c>
-      <s:c r="E5" s="1" t="n">
+      <s:c r="E5" s="2" t="n">
         <s:v>80</s:v>
       </s:c>
-      <s:c r="F5" s="1" t="inlineStr">
+      <s:c r="F5" s="2" t="inlineStr">
         <s:is>
           <s:t>{Type=Item,Id=105,Count=1}</s:t>
         </s:is>
       </s:c>
-      <s:c r="G5" s="1" t="inlineStr">
+      <s:c r="G5" s="2" t="inlineStr">
         <s:is>
           <s:t>15 分钟力量卡</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="6" ht="27" customHeight="1" s="2">
-      <s:c r="A6" s="1" t="n">
+    <s:row r="6" ht="27" customHeight="1" s="1">
+      <s:c r="A6" s="2" t="n">
         <s:v>3</s:v>
       </s:c>
-      <s:c r="B6" s="1" t="inlineStr">
+      <s:c r="B6" s="2" t="inlineStr">
         <s:is>
           <s:t>OnlineTime</s:t>
         </s:is>
@@ -1471,25 +1471,25 @@
           <s:t>Stay online for 30 minutes</s:t>
         </s:is>
       </s:c>
-      <s:c r="E6" s="1" t="n">
+      <s:c r="E6" s="2" t="n">
         <s:v>30</s:v>
       </s:c>
-      <s:c r="F6" s="1" t="inlineStr">
+      <s:c r="F6" s="2" t="inlineStr">
         <s:is>
           <s:t>{Type=Gem, Count=5}</s:t>
         </s:is>
       </s:c>
-      <s:c r="G6" s="1" t="inlineStr">
+      <s:c r="G6" s="2" t="inlineStr">
         <s:is>
           <s:t>4钻石</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="7">
-      <s:c r="A7" s="1" t="n">
+      <s:c r="A7" s="2" t="n">
         <s:v>4</s:v>
       </s:c>
-      <s:c r="B7" s="1" t="inlineStr">
+      <s:c r="B7" s="2" t="inlineStr">
         <s:is>
           <s:t>GetDog</s:t>
         </s:is>
@@ -1504,25 +1504,25 @@
           <s:t>Pick up 10 dogs</s:t>
         </s:is>
       </s:c>
-      <s:c r="E7" s="1" t="n">
+      <s:c r="E7" s="2" t="n">
         <s:v>10</s:v>
       </s:c>
-      <s:c r="F7" s="1" t="inlineStr">
+      <s:c r="F7" s="2" t="inlineStr">
         <s:is>
           <s:t>{Type=Gem, Count=3}</s:t>
         </s:is>
       </s:c>
-      <s:c r="G7" s="1" t="inlineStr">
+      <s:c r="G7" s="2" t="inlineStr">
         <s:is>
           <s:t>3钻石</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="8" ht="27" customHeight="1" s="2">
-      <s:c r="A8" s="1" t="n">
+    <s:row r="8" ht="27" customHeight="1" s="1">
+      <s:c r="A8" s="2" t="n">
         <s:v>5</s:v>
       </s:c>
-      <s:c r="B8" s="1" t="inlineStr">
+      <s:c r="B8" s="2" t="inlineStr">
         <s:is>
           <s:t>ForFriendPlay</s:t>
         </s:is>
@@ -1537,15 +1537,15 @@
           <s:t>Be in the same room as 2 friends</s:t>
         </s:is>
       </s:c>
-      <s:c r="E8" s="1" t="n">
+      <s:c r="E8" s="2" t="n">
         <s:v>2</s:v>
       </s:c>
-      <s:c r="F8" s="1" t="inlineStr">
+      <s:c r="F8" s="2" t="inlineStr">
         <s:is>
           <s:t>{Type=Gem, Count=2}</s:t>
         </s:is>
       </s:c>
-      <s:c r="G8" s="1" t="inlineStr">
+      <s:c r="G8" s="2" t="inlineStr">
         <s:is>
           <s:t>3钻石</s:t>
         </s:is>
@@ -1565,80 +1565,80 @@
   <s:dimension ref="A1:E10"/>
   <s:sheetFormatPr baseColWidth="8" defaultColWidth="8.891666666666669" defaultRowHeight="13.5" outlineLevelCol="4"/>
   <s:cols>
-    <s:col width="30.85" customWidth="1" style="2" min="2" max="2"/>
-    <s:col width="34.2833333333333" customWidth="1" style="2" min="3" max="3"/>
-    <s:col width="28.7583333333333" customWidth="1" style="2" min="4" max="4"/>
-    <s:col width="23.3583333333333" customWidth="1" style="2" min="5" max="5"/>
+    <s:col width="30.85" customWidth="1" style="1" min="2" max="2"/>
+    <s:col width="34.2833333333333" customWidth="1" style="1" min="3" max="3"/>
+    <s:col width="28.7583333333333" customWidth="1" style="1" min="4" max="4"/>
+    <s:col width="23.3583333333333" customWidth="1" style="1" min="5" max="5"/>
   </s:cols>
   <s:sheetData>
     <s:row r="1">
-      <s:c r="A1" s="1" t="inlineStr">
+      <s:c r="A1" s="2" t="inlineStr">
         <s:is>
           <s:t>等级</s:t>
         </s:is>
       </s:c>
-      <s:c r="B1" s="1" t="inlineStr">
+      <s:c r="B1" s="2" t="inlineStr">
         <s:is>
           <s:t>需要消费的金额</s:t>
         </s:is>
       </s:c>
-      <s:c r="C1" s="1" t="inlineStr">
+      <s:c r="C1" s="2" t="inlineStr">
         <s:is>
           <s:t>s</s:t>
         </s:is>
       </s:c>
-      <s:c r="D1" s="1" t="inlineStr">
+      <s:c r="D1" s="2" t="inlineStr">
         <s:is>
           <s:t>奖励</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="2">
-      <s:c r="A2" s="1" t="inlineStr">
+      <s:c r="A2" s="2" t="inlineStr">
         <s:is>
           <s:t>Index</s:t>
         </s:is>
       </s:c>
-      <s:c r="B2" s="1" t="inlineStr">
+      <s:c r="B2" s="2" t="inlineStr">
         <s:is>
           <s:t>LoginDays</s:t>
         </s:is>
       </s:c>
-      <s:c r="C2" s="1" t="inlineStr">
+      <s:c r="C2" s="2" t="inlineStr">
         <s:is>
           <s:t>Desc</s:t>
         </s:is>
       </s:c>
-      <s:c r="D2" s="1" t="inlineStr">
+      <s:c r="D2" s="2" t="inlineStr">
         <s:is>
           <s:t>Reward</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="3" ht="14.25" customHeight="1" s="2">
-      <s:c r="A3" s="1" t="inlineStr">
+    <s:row r="3" ht="14.25" customHeight="1" s="1">
+      <s:c r="A3" s="2" t="inlineStr">
         <s:is>
           <s:t>number</s:t>
         </s:is>
       </s:c>
-      <s:c r="B3" s="1" t="inlineStr">
+      <s:c r="B3" s="2" t="inlineStr">
         <s:is>
           <s:t>number</s:t>
         </s:is>
       </s:c>
-      <s:c r="C3" s="1" t="inlineStr">
+      <s:c r="C3" s="2" t="inlineStr">
         <s:is>
           <s:t>string</s:t>
         </s:is>
       </s:c>
-      <s:c r="D3" s="1" t="inlineStr">
+      <s:c r="D3" s="2" t="inlineStr">
         <s:is>
           <s:t>kv_string</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="4" ht="23.25" customHeight="1" s="2">
-      <s:c r="A4" s="1" t="n">
+    <s:row r="4" ht="23.25" customHeight="1" s="1">
+      <s:c r="A4" s="2" t="n">
         <s:v>1</s:v>
       </s:c>
       <s:c r="B4" s="3" t="n">
@@ -1649,15 +1649,15 @@
           <s:t>背包扩容卡X1</s:t>
         </s:is>
       </s:c>
-      <s:c r="D4" s="1" t="inlineStr">
+      <s:c r="D4" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=104,Count=1</s:t>
         </s:is>
       </s:c>
       <s:c r="E4" s="5" t="n"/>
     </s:row>
-    <s:row r="5" ht="23.25" customHeight="1" s="2">
-      <s:c r="A5" s="1" t="n">
+    <s:row r="5" ht="23.25" customHeight="1" s="1">
+      <s:c r="A5" s="2" t="n">
         <s:v>2</s:v>
       </s:c>
       <s:c r="B5" s="3" t="n">
@@ -1668,15 +1668,15 @@
           <s:t>15钻石</s:t>
         </s:is>
       </s:c>
-      <s:c r="D5" s="1" t="inlineStr">
+      <s:c r="D5" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Gem, Count=15</s:t>
         </s:is>
       </s:c>
       <s:c r="E5" s="5" t="n"/>
     </s:row>
-    <s:row r="6" ht="14.25" customHeight="1" s="2">
-      <s:c r="A6" s="1" t="n">
+    <s:row r="6" ht="14.25" customHeight="1" s="1">
+      <s:c r="A6" s="2" t="n">
         <s:v>3</s:v>
       </s:c>
       <s:c r="B6" s="3" t="n">
@@ -1687,15 +1687,15 @@
           <s:t>双倍出售卡X3</s:t>
         </s:is>
       </s:c>
-      <s:c r="D6" s="1" t="inlineStr">
+      <s:c r="D6" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=103,Count=3</s:t>
         </s:is>
       </s:c>
-      <s:c r="E6" s="1" t="n"/>
-    </s:row>
-    <s:row r="7" ht="23" customHeight="1" s="2">
-      <s:c r="A7" s="1" t="n">
+      <s:c r="E6" s="2" t="n"/>
+    </s:row>
+    <s:row r="7" ht="23" customHeight="1" s="1">
+      <s:c r="A7" s="2" t="n">
         <s:v>4</s:v>
       </s:c>
       <s:c r="B7" s="3" t="n">
@@ -1706,15 +1706,15 @@
           <s:t>30分钟力量卡X2</s:t>
         </s:is>
       </s:c>
-      <s:c r="D7" s="1" t="inlineStr">
+      <s:c r="D7" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=106,Count=2</s:t>
         </s:is>
       </s:c>
       <s:c r="E7" s="5" t="n"/>
     </s:row>
-    <s:row r="8" ht="23.25" customHeight="1" s="2">
-      <s:c r="A8" s="1" t="n">
+    <s:row r="8" ht="23.25" customHeight="1" s="1">
+      <s:c r="A8" s="2" t="n">
         <s:v>5</s:v>
       </s:c>
       <s:c r="B8" s="3" t="n">
@@ -1725,15 +1725,15 @@
           <s:t>15钻石</s:t>
         </s:is>
       </s:c>
-      <s:c r="D8" s="1" t="inlineStr">
+      <s:c r="D8" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Gem, Count=15</s:t>
         </s:is>
       </s:c>
       <s:c r="E8" s="6" t="n"/>
     </s:row>
-    <s:row r="9" ht="14.25" customHeight="1" s="2">
-      <s:c r="A9" s="1" t="n">
+    <s:row r="9" ht="14.25" customHeight="1" s="1">
+      <s:c r="A9" s="2" t="n">
         <s:v>6</s:v>
       </s:c>
       <s:c r="B9" s="3" t="n">
@@ -1744,14 +1744,14 @@
           <s:t>背包扩容卡X2</s:t>
         </s:is>
       </s:c>
-      <s:c r="D9" s="1" t="inlineStr">
+      <s:c r="D9" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=104,Count=2</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="10" ht="14.25" customHeight="1" s="2">
-      <s:c r="A10" s="1" t="n">
+    <s:row r="10" ht="14.25" customHeight="1" s="1">
+      <s:c r="A10" s="2" t="n">
         <s:v>7</s:v>
       </s:c>
       <s:c r="B10" s="3" t="n">
@@ -1762,7 +1762,7 @@
           <s:t>20钻石</s:t>
         </s:is>
       </s:c>
-      <s:c r="D10" s="1" t="inlineStr">
+      <s:c r="D10" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Gem, Count=20</s:t>
         </s:is>
@@ -1782,254 +1782,254 @@
   <s:dimension ref="A1:D13"/>
   <s:sheetFormatPr baseColWidth="8" defaultColWidth="8.891666666666669" defaultRowHeight="13.5" outlineLevelCol="3"/>
   <s:cols>
-    <s:col width="9" customWidth="1" style="2" min="1" max="1"/>
-    <s:col width="23.325" customWidth="1" style="2" min="2" max="2"/>
-    <s:col width="19.4166666666667" customWidth="1" style="2" min="3" max="3"/>
-    <s:col width="38.6166666666667" customWidth="1" style="2" min="4" max="4"/>
-    <s:col width="9" customWidth="1" style="2" min="5" max="16384"/>
+    <s:col width="9" customWidth="1" style="1" min="1" max="1"/>
+    <s:col width="23.325" customWidth="1" style="1" min="2" max="2"/>
+    <s:col width="19.4166666666667" customWidth="1" style="1" min="3" max="3"/>
+    <s:col width="38.6166666666667" customWidth="1" style="1" min="4" max="4"/>
+    <s:col width="9" customWidth="1" style="1" min="5" max="16384"/>
   </s:cols>
   <s:sheetData>
-    <s:row r="1" customFormat="1" s="1">
-      <s:c r="A1" s="1" t="inlineStr">
+    <s:row r="1" customFormat="1" s="2">
+      <s:c r="A1" s="2" t="inlineStr">
         <s:is>
           <s:t>索引</s:t>
         </s:is>
       </s:c>
-      <s:c r="B1" s="1" t="inlineStr">
+      <s:c r="B1" s="2" t="inlineStr">
         <s:is>
           <s:t>时长</s:t>
         </s:is>
       </s:c>
-      <s:c r="C1" s="1" t="inlineStr">
+      <s:c r="C1" s="2" t="inlineStr">
         <s:is>
           <s:t>描述</s:t>
         </s:is>
       </s:c>
-      <s:c r="D1" s="1" t="inlineStr">
+      <s:c r="D1" s="2" t="inlineStr">
         <s:is>
           <s:t>奖励</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="2" customFormat="1" s="1">
-      <s:c r="A2" s="1" t="inlineStr">
+    <s:row r="2" customFormat="1" s="2">
+      <s:c r="A2" s="2" t="inlineStr">
         <s:is>
           <s:t>Index</s:t>
         </s:is>
       </s:c>
-      <s:c r="B2" s="1" t="inlineStr">
+      <s:c r="B2" s="2" t="inlineStr">
         <s:is>
           <s:t>TargetMinutes</s:t>
         </s:is>
       </s:c>
-      <s:c r="C2" s="1" t="inlineStr">
+      <s:c r="C2" s="2" t="inlineStr">
         <s:is>
           <s:t>Desc</s:t>
         </s:is>
       </s:c>
-      <s:c r="D2" s="1" t="inlineStr">
+      <s:c r="D2" s="2" t="inlineStr">
         <s:is>
           <s:t>Reward</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="3" customFormat="1" s="1">
-      <s:c r="A3" s="1" t="inlineStr">
+    <s:row r="3" customFormat="1" s="2">
+      <s:c r="A3" s="2" t="inlineStr">
         <s:is>
           <s:t>number</s:t>
         </s:is>
       </s:c>
-      <s:c r="B3" s="1" t="inlineStr">
+      <s:c r="B3" s="2" t="inlineStr">
         <s:is>
           <s:t>number</s:t>
         </s:is>
       </s:c>
-      <s:c r="C3" s="1" t="inlineStr">
+      <s:c r="C3" s="2" t="inlineStr">
         <s:is>
           <s:t>string</s:t>
         </s:is>
       </s:c>
-      <s:c r="D3" s="1" t="inlineStr">
+      <s:c r="D3" s="2" t="inlineStr">
         <s:is>
           <s:t>kv_string</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="4" customFormat="1" s="1">
-      <s:c r="A4" s="1" t="n">
+    <s:row r="4" customFormat="1" s="2">
+      <s:c r="A4" s="2" t="n">
         <s:v>1</s:v>
       </s:c>
-      <s:c r="B4" s="1" t="n">
+      <s:c r="B4" s="2" t="n">
         <s:v>5</s:v>
       </s:c>
-      <s:c r="C4" s="1" t="inlineStr">
+      <s:c r="C4" s="2" t="inlineStr">
         <s:is>
           <s:t>NPC卡X2</s:t>
         </s:is>
       </s:c>
-      <s:c r="D4" s="1" t="inlineStr">
+      <s:c r="D4" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=107,Count=2</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="5" customFormat="1" s="1">
-      <s:c r="A5" s="1" t="n">
+    <s:row r="5" customFormat="1" s="2">
+      <s:c r="A5" s="2" t="n">
         <s:v>2</s:v>
       </s:c>
-      <s:c r="B5" s="1" t="n">
+      <s:c r="B5" s="2" t="n">
         <s:v>10</s:v>
       </s:c>
-      <s:c r="C5" s="1" t="inlineStr">
+      <s:c r="C5" s="2" t="inlineStr">
         <s:is>
           <s:t>15分钟力量卡</s:t>
         </s:is>
       </s:c>
-      <s:c r="D5" s="1" t="inlineStr">
+      <s:c r="D5" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=105,Count=1</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="6" customFormat="1" s="1">
-      <s:c r="A6" s="1" t="n">
+    <s:row r="6" customFormat="1" s="2">
+      <s:c r="A6" s="2" t="n">
         <s:v>3</s:v>
       </s:c>
-      <s:c r="B6" s="1" t="n">
+      <s:c r="B6" s="2" t="n">
         <s:v>20</s:v>
       </s:c>
-      <s:c r="C6" s="1" t="inlineStr">
+      <s:c r="C6" s="2" t="inlineStr">
         <s:is>
           <s:t>双倍出售卡X1</s:t>
         </s:is>
       </s:c>
-      <s:c r="D6" s="1" t="inlineStr">
+      <s:c r="D6" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=103,Count=1</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="7" customFormat="1" s="1">
-      <s:c r="A7" s="1" t="n">
+    <s:row r="7" customFormat="1" s="2">
+      <s:c r="A7" s="2" t="n">
         <s:v>4</s:v>
       </s:c>
-      <s:c r="B7" s="1" t="n">
+      <s:c r="B7" s="2" t="n">
         <s:v>25</s:v>
       </s:c>
-      <s:c r="C7" s="1" t="inlineStr">
+      <s:c r="C7" s="2" t="inlineStr">
         <s:is>
           <s:t>2钻石</s:t>
         </s:is>
       </s:c>
-      <s:c r="D7" s="1" t="inlineStr">
+      <s:c r="D7" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Gem, Count=2</s:t>
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="8" customFormat="1" s="1">
-      <s:c r="A8" s="1" t="n">
+    <s:row r="8" customFormat="1" s="2">
+      <s:c r="A8" s="2" t="n">
         <s:v>5</s:v>
       </s:c>
-      <s:c r="B8" s="1" t="n">
+      <s:c r="B8" s="2" t="n">
         <s:v>35</s:v>
       </s:c>
-      <s:c r="C8" s="1" t="inlineStr">
+      <s:c r="C8" s="2" t="inlineStr">
         <s:is>
           <s:t>30分钟力量卡X1</s:t>
         </s:is>
       </s:c>
-      <s:c r="D8" s="1" t="inlineStr">
+      <s:c r="D8" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=106,Count=1</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="9">
-      <s:c r="A9" s="1" t="n">
+      <s:c r="A9" s="2" t="n">
         <s:v>6</s:v>
       </s:c>
-      <s:c r="B9" s="1" t="n">
+      <s:c r="B9" s="2" t="n">
         <s:v>45</s:v>
       </s:c>
-      <s:c r="C9" s="1" t="inlineStr">
+      <s:c r="C9" s="2" t="inlineStr">
         <s:is>
           <s:t>3钻石</s:t>
         </s:is>
       </s:c>
-      <s:c r="D9" s="1" t="inlineStr">
+      <s:c r="D9" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Gem, Count=3</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="10">
-      <s:c r="A10" s="1" t="n">
+      <s:c r="A10" s="2" t="n">
         <s:v>7</s:v>
       </s:c>
-      <s:c r="B10" s="1" t="n">
+      <s:c r="B10" s="2" t="n">
         <s:v>55</s:v>
       </s:c>
-      <s:c r="C10" s="1" t="inlineStr">
+      <s:c r="C10" s="2" t="inlineStr">
         <s:is>
           <s:t>背包扩容卡(一小时)</s:t>
         </s:is>
       </s:c>
-      <s:c r="D10" s="1" t="inlineStr">
+      <s:c r="D10" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=104,Count=1</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="11">
-      <s:c r="A11" s="1" t="n">
+      <s:c r="A11" s="2" t="n">
         <s:v>8</s:v>
       </s:c>
-      <s:c r="B11" s="1" t="n">
+      <s:c r="B11" s="2" t="n">
         <s:v>65</s:v>
       </s:c>
-      <s:c r="C11" s="1" t="inlineStr">
+      <s:c r="C11" s="2" t="inlineStr">
         <s:is>
           <s:t>5钻石</s:t>
         </s:is>
       </s:c>
-      <s:c r="D11" s="1" t="inlineStr">
+      <s:c r="D11" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Gem, Count=5</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="12">
-      <s:c r="A12" s="1" t="n">
+      <s:c r="A12" s="2" t="n">
         <s:v>9</s:v>
       </s:c>
-      <s:c r="B12" s="1" t="n">
+      <s:c r="B12" s="2" t="n">
         <s:v>75</s:v>
       </s:c>
-      <s:c r="C12" s="1" t="inlineStr">
+      <s:c r="C12" s="2" t="inlineStr">
         <s:is>
           <s:t>双倍出售卡X1</s:t>
         </s:is>
       </s:c>
-      <s:c r="D12" s="1" t="inlineStr">
+      <s:c r="D12" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=103,Count=1</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="13">
-      <s:c r="A13" s="1" t="n">
+      <s:c r="A13" s="2" t="n">
         <s:v>10</s:v>
       </s:c>
-      <s:c r="B13" s="1" t="n">
+      <s:c r="B13" s="2" t="n">
         <s:v>90</s:v>
       </s:c>
-      <s:c r="C13" s="1" t="inlineStr">
+      <s:c r="C13" s="2" t="inlineStr">
         <s:is>
           <s:t>30分钟力量卡X1</s:t>
         </s:is>
       </s:c>
-      <s:c r="D13" s="1" t="inlineStr">
+      <s:c r="D13" s="2" t="inlineStr">
         <s:is>
           <s:t>Type=Item,Id=106,Count=1</s:t>
         </s:is>
@@ -2047,10 +2047,11 @@
     <s:pageSetUpPr/>
   </s:sheetPr>
   <s:dimension ref="A1:D3"/>
-  <s:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="2"/>
+  <s:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="3"/>
   <s:cols>
-    <s:col width="44.5" customWidth="1" style="2" min="1" max="1"/>
-    <s:col width="37" customWidth="1" style="2" min="2" max="2"/>
+    <s:col width="44.5" customWidth="1" style="1" min="1" max="1"/>
+    <s:col width="37" customWidth="1" style="1" min="2" max="2"/>
+    <s:col width="23" customWidth="1" style="1" min="3" max="3"/>
   </s:cols>
   <s:sheetData>
     <s:row r="1">
@@ -2091,27 +2092,29 @@
       </s:c>
       <s:c r="D2" s="0" t="inlineStr">
         <s:is>
-          <s:t>触发时长，单位：分钟。按当天累计在线时长计算，重进保留、UTC 零点重置。达到本值且引用奖励已解锁、未领取时，按 ESC 显示中央礼包，左侧提示可立即领取；关闭系统菜单后可点击领取。若引用奖励的 TargetMinutes 更大，须同时达到该门槛。</s:t>
+          <s:t>提示期限，单位：分钟。默认 5 表示本次进服后的前 5 分钟内按 ESC 即可显示，未满 5 分钟就能领取，不是在线满 5 分钟才解锁；达到 5 分钟后不再显示或领取。重登按新会话重新计时，但已经领取的玩家永久不再获得。符合条件时，显示礼包前先 Close 主界面 Main 以外的所有游戏弹窗，等关闭完成再显示礼包；系统 ESC 菜单保留。</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="3">
       <s:c r="A3" s="0" t="inlineStr">
         <s:is>
-          <s:t>string,number</s:t>
+          <s:t>string,kv_string</s:t>
         </s:is>
       </s:c>
       <s:c r="B3" s="0" t="inlineStr">
         <s:is>
-          <s:t>OnlineRewardId</s:t>
-        </s:is>
-      </s:c>
-      <s:c r="C3" s="0" t="n">
-        <s:v>1</s:v>
+          <s:t>Reward</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C3" s="0" t="inlineStr">
+        <s:is>
+          <s:t>Type=Item,Id=107,Count=2</s:t>
+        </s:is>
       </s:c>
       <s:c r="D3" s="0" t="inlineStr">
         <s:is>
-          <s:t>引用 OnlineRewardData 页签的 Index，必须填写存在的奖励编号。奖励解锁分钟数在该行 TargetMinutes 修改；奖励类型、道具 ID、数量在 Reward 修改：Type=Item,Id=107,Count=2 表示 107 号道具 2 个；Type=Gem,Count=5 表示 5 钻石。与福利页共享每天一次的领取资格，任一处领取后均不可重复领取；背包不足不消耗资格。</s:t>
+          <s:t>本一次性礼包的独立奖励。Type=Item,Id=107,Count=2 表示 107 号道具 2 个；Type=Gem,Count=5 表示 5 钻石。每个玩家永久只能领取一次，跨天、重登、重生都不重置；与每日在线奖励的领取记录互不影响，发奖失败不消耗资格，可在本次提示期限内重试。</s:t>
         </s:is>
       </s:c>
     </s:row>

</xml_diff>